<commit_message>
Updated on 10-22-2023 at 07:53
</commit_message>
<xml_diff>
--- a/output/accuracy.xlsx
+++ b/output/accuracy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\home\gustavo\LOVO\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFF46AC1-A0AA-4843-864F-B95BB5D5227B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2EE63A9-6836-4974-821A-B2BB4175488E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="2115" yWindow="2115" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -33,11 +33,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -75,12 +70,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -91,9 +83,12 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FFFF5050"/>
-      <color rgb="FFFF6600"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FFFD6B6B"/>
+      <color rgb="FFFF5D5D"/>
+      <color rgb="FFFF7D7D"/>
+      <color rgb="FFE75F5F"/>
+      <color rgb="FF37A9FF"/>
+      <color rgb="FF62BE71"/>
     </mruColors>
   </colors>
   <extLst>
@@ -396,43 +391,46 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B1" s="1">
+        <v>0</v>
+      </c>
       <c r="C1" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D1" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E1" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F1" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G1" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H1" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I1" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J1" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K1" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L1" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0</v>
       </c>
-      <c r="B2" s="2">
-        <v>5</v>
+      <c r="B2">
+        <v>1</v>
       </c>
       <c r="C2">
         <v>15.23</v>
@@ -469,8 +467,8 @@
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="2">
-        <v>6</v>
+      <c r="B3">
+        <v>2</v>
       </c>
       <c r="C3">
         <v>13.32</v>
@@ -507,8 +505,8 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="2">
-        <v>7</v>
+      <c r="B4">
+        <v>3</v>
       </c>
       <c r="C4">
         <v>3.17</v>
@@ -545,8 +543,8 @@
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="2">
-        <v>8</v>
+      <c r="B5">
+        <v>4</v>
       </c>
       <c r="C5">
         <v>0.2</v>
@@ -583,8 +581,8 @@
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="2">
-        <v>9</v>
+      <c r="B6">
+        <v>5</v>
       </c>
       <c r="C6">
         <v>0.18</v>
@@ -621,8 +619,8 @@
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="2">
-        <v>10</v>
+      <c r="B7">
+        <v>6</v>
       </c>
       <c r="C7">
         <v>0.13</v>
@@ -659,8 +657,8 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="2">
-        <v>11</v>
+      <c r="B8">
+        <v>7</v>
       </c>
       <c r="C8">
         <v>0.16</v>
@@ -697,8 +695,8 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="2">
-        <v>12</v>
+      <c r="B9">
+        <v>8</v>
       </c>
       <c r="C9">
         <v>0.28999999999999998</v>
@@ -735,8 +733,8 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="2">
-        <v>13</v>
+      <c r="B10">
+        <v>9</v>
       </c>
       <c r="C10">
         <v>0.2</v>
@@ -773,8 +771,8 @@
       <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="B11" s="2">
-        <v>14</v>
+      <c r="B11">
+        <v>10</v>
       </c>
       <c r="C11">
         <v>0.91</v>
@@ -811,8 +809,8 @@
       <c r="A12" s="1">
         <v>10</v>
       </c>
-      <c r="B12" s="2">
-        <v>15</v>
+      <c r="B12">
+        <v>11</v>
       </c>
       <c r="C12">
         <v>1.43</v>
@@ -849,8 +847,8 @@
       <c r="A13" s="1">
         <v>11</v>
       </c>
-      <c r="B13" s="2">
-        <v>16</v>
+      <c r="B13">
+        <v>12</v>
       </c>
       <c r="C13">
         <v>1.77</v>
@@ -887,8 +885,8 @@
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="2">
-        <v>17</v>
+      <c r="B14">
+        <v>13</v>
       </c>
       <c r="C14">
         <v>2.04</v>
@@ -925,8 +923,8 @@
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="2">
-        <v>18</v>
+      <c r="B15">
+        <v>14</v>
       </c>
       <c r="C15">
         <v>2.33</v>
@@ -963,8 +961,8 @@
       <c r="A16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="2">
-        <v>19</v>
+      <c r="B16">
+        <v>15</v>
       </c>
       <c r="C16">
         <v>2.4500000000000002</v>
@@ -1001,8 +999,8 @@
       <c r="A17" s="1">
         <v>15</v>
       </c>
-      <c r="B17" s="2">
-        <v>20</v>
+      <c r="B17">
+        <v>16</v>
       </c>
       <c r="C17">
         <v>2.42</v>
@@ -1039,8 +1037,8 @@
       <c r="A18" s="1">
         <v>16</v>
       </c>
-      <c r="B18" s="2">
-        <v>21</v>
+      <c r="B18">
+        <v>17</v>
       </c>
       <c r="C18">
         <v>2.46</v>
@@ -1077,8 +1075,8 @@
       <c r="A19" s="1">
         <v>17</v>
       </c>
-      <c r="B19" s="2">
-        <v>22</v>
+      <c r="B19">
+        <v>18</v>
       </c>
       <c r="C19">
         <v>2.13</v>
@@ -1115,8 +1113,8 @@
       <c r="A20" s="1">
         <v>18</v>
       </c>
-      <c r="B20" s="2">
-        <v>23</v>
+      <c r="B20">
+        <v>19</v>
       </c>
       <c r="C20">
         <v>2.2599999999999998</v>
@@ -1153,8 +1151,8 @@
       <c r="A21" s="1">
         <v>19</v>
       </c>
-      <c r="B21" s="2">
-        <v>24</v>
+      <c r="B21">
+        <v>20</v>
       </c>
       <c r="C21">
         <v>2.29</v>
@@ -1191,8 +1189,8 @@
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" s="2">
-        <v>25</v>
+      <c r="B22">
+        <v>21</v>
       </c>
       <c r="C22">
         <v>2.2400000000000002</v>
@@ -1229,8 +1227,8 @@
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" s="2">
-        <v>26</v>
+      <c r="B23">
+        <v>22</v>
       </c>
       <c r="C23">
         <v>2.2400000000000002</v>
@@ -1267,8 +1265,8 @@
       <c r="A24" s="1">
         <v>22</v>
       </c>
-      <c r="B24" s="2">
-        <v>27</v>
+      <c r="B24">
+        <v>23</v>
       </c>
       <c r="C24">
         <v>2.23</v>
@@ -1305,8 +1303,8 @@
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" s="2">
-        <v>28</v>
+      <c r="B25">
+        <v>24</v>
       </c>
       <c r="C25">
         <v>2.79</v>
@@ -1343,8 +1341,8 @@
       <c r="A26" s="1">
         <v>24</v>
       </c>
-      <c r="B26" s="2">
-        <v>29</v>
+      <c r="B26">
+        <v>25</v>
       </c>
       <c r="C26">
         <v>2.57</v>
@@ -1381,8 +1379,8 @@
       <c r="A27" s="1">
         <v>25</v>
       </c>
-      <c r="B27" s="2">
-        <v>30</v>
+      <c r="B27">
+        <v>26</v>
       </c>
       <c r="C27">
         <v>2.75</v>
@@ -1417,90 +1415,27 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:L27">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="20"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="FF62BE71"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFE75F5F"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="20"/>
         <cfvo type="num" val="100"/>
-        <color theme="0"/>
-        <color theme="4"/>
-        <color rgb="FFFF5050"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percent" val="50"/>
-        <cfvo type="percent" val="100"/>
-        <color theme="0"/>
-        <color theme="3" tint="0.39997558519241921"/>
-        <color rgb="FFFF5050"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="30"/>
-        <cfvo type="num" val="60"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="30"/>
-        <cfvo type="num" val="60"/>
         <color theme="3" tint="0.59999389629810485"/>
-        <color rgb="FFFFFF00"/>
-        <color theme="9" tint="-0.249977111117893"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="100"/>
-        <color theme="4"/>
-        <color rgb="FFFF6600"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color theme="4"/>
-        <color rgb="FFFF5050"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="100"/>
-        <color rgb="FFFF7128"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percent" val="100"/>
-        <color theme="3" tint="0.59999389629810485"/>
-        <color rgb="FFFF5050"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFFD6B6B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>